<commit_message>
Regenerate ils-postplanner-2026-04-27.xlsx (test run artifact)
Re-generated during April 28 pipeline session when testing PostPlanner format compatibility.

https://claude.ai/code/session_019iWqrzRsXtYnUAzDWh37Q2
</commit_message>
<xml_diff>
--- a/Softball/postplanner-imports/ils-postplanner-2026-04-27.xlsx
+++ b/Softball/postplanner-imports/ils-postplanner-2026-04-27.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/27/2026  11:09</t>
+          <t>04/27/2026  09:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,7 +494,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/27/2026  12:21</t>
+          <t>04/27/2026  09:05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -509,7 +509,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/27/2026  13:33</t>
+          <t>04/27/2026  11:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -524,7 +524,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/27/2026  14:45</t>
+          <t>04/27/2026  11:05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -539,7 +539,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/27/2026  15:57</t>
+          <t>04/27/2026  13:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/27/2026  17:09</t>
+          <t>04/27/2026  15:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -575,7 +575,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/27/2026  18:21</t>
+          <t>04/27/2026  15:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -590,7 +590,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/27/2026  19:33</t>
+          <t>04/27/2026  17:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -606,7 +606,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04/27/2026  20:45</t>
+          <t>04/27/2026  20:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">

</xml_diff>